<commit_message>
クラス図 (users) 更新 2025.10.10
</commit_message>
<xml_diff>
--- a/class_diagram/users/クラス図_面談予約sys (users)_最新.xlsx
+++ b/class_diagram/users/クラス図_面談予約sys (users)_最新.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ktc\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="32" documentId="13_ncr:1_{DDC5F448-C290-4053-AF89-2C5F4DE0E5F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0C72D9F3-5572-446B-8968-DAF69F875519}"/>
+  <xr:revisionPtr revIDLastSave="39" documentId="13_ncr:1_{DDC5F448-C290-4053-AF89-2C5F4DE0E5F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{19934BFF-BE7A-41D8-9B45-42D3196BAEB8}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="18945" windowHeight="11190" firstSheet="18" activeTab="21" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="18945" windowHeight="11190" firstSheet="21" activeTab="29" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="controller.UserPreServlet" sheetId="1" r:id="rId1"/>
@@ -39,6 +39,10 @@
     <sheet name="dao.PastGetDAO" sheetId="22" r:id="rId24"/>
     <sheet name="controller.EmailSendPreServlet" sheetId="23" r:id="rId25"/>
     <sheet name="dao.EmailCheckDAO" sheetId="24" r:id="rId26"/>
+    <sheet name="dao.StatusGetDAO" sheetId="32" r:id="rId27"/>
+    <sheet name="controller.StatusGetServlet" sheetId="33" r:id="rId28"/>
+    <sheet name="controller.WeeksGet" sheetId="34" r:id="rId29"/>
+    <sheet name="controller.DatesGet" sheetId="35" r:id="rId30"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -7629,6 +7633,2202 @@
             </a:solidFill>
             <a:latin typeface="Aptos Narrow" panose="020B0004020202020204" pitchFamily="34" charset="0"/>
           </a:endParaRPr>
+        </a:p>
+        <a:p>
+          <a:pPr marL="0" marR="0" indent="0" algn="l">
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+            <a:spcBef>
+              <a:spcPts val="0"/>
+            </a:spcBef>
+            <a:spcAft>
+              <a:spcPts val="0"/>
+            </a:spcAft>
+          </a:pPr>
+          <a:endParaRPr lang="en-US" sz="1100" b="0" i="0" u="none" strike="noStrike">
+            <a:solidFill>
+              <a:schemeClr val="lt1"/>
+            </a:solidFill>
+            <a:latin typeface="Aptos Narrow" panose="020B0004020202020204" pitchFamily="34" charset="0"/>
+          </a:endParaRPr>
+        </a:p>
+        <a:p>
+          <a:pPr marL="0" marR="0" indent="0" algn="l">
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+            <a:spcBef>
+              <a:spcPts val="0"/>
+            </a:spcBef>
+            <a:spcAft>
+              <a:spcPts val="0"/>
+            </a:spcAft>
+          </a:pPr>
+          <a:endParaRPr lang="en-US" sz="1100" b="0" i="0" u="none" strike="noStrike">
+            <a:solidFill>
+              <a:schemeClr val="lt1"/>
+            </a:solidFill>
+            <a:latin typeface="Aptos Narrow" panose="020B0004020202020204" pitchFamily="34" charset="0"/>
+          </a:endParaRPr>
+        </a:p>
+        <a:p>
+          <a:pPr marL="0" marR="0" indent="0" algn="l">
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+            <a:spcBef>
+              <a:spcPts val="0"/>
+            </a:spcBef>
+            <a:spcAft>
+              <a:spcPts val="0"/>
+            </a:spcAft>
+          </a:pPr>
+          <a:endParaRPr lang="en-US" sz="1100" b="0" i="0" u="none" strike="noStrike">
+            <a:solidFill>
+              <a:schemeClr val="lt1"/>
+            </a:solidFill>
+            <a:latin typeface="Aptos Narrow" panose="020B0004020202020204" pitchFamily="34" charset="0"/>
+          </a:endParaRPr>
+        </a:p>
+        <a:p>
+          <a:pPr marL="0" marR="0" indent="0" algn="l">
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+            <a:spcBef>
+              <a:spcPts val="0"/>
+            </a:spcBef>
+            <a:spcAft>
+              <a:spcPts val="0"/>
+            </a:spcAft>
+          </a:pPr>
+          <a:endParaRPr lang="en-US" sz="1100" b="0" i="0" u="none" strike="noStrike">
+            <a:solidFill>
+              <a:schemeClr val="lt1"/>
+            </a:solidFill>
+            <a:latin typeface="Aptos Narrow" panose="020B0004020202020204" pitchFamily="34" charset="0"/>
+          </a:endParaRPr>
+        </a:p>
+        <a:p>
+          <a:pPr marL="0" marR="0" indent="0" algn="l">
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+            <a:spcBef>
+              <a:spcPts val="0"/>
+            </a:spcBef>
+            <a:spcAft>
+              <a:spcPts val="0"/>
+            </a:spcAft>
+          </a:pPr>
+          <a:endParaRPr lang="en-US" sz="1100" b="0" i="0" u="none" strike="noStrike">
+            <a:solidFill>
+              <a:schemeClr val="lt1"/>
+            </a:solidFill>
+            <a:latin typeface="Aptos Narrow" panose="020B0004020202020204" pitchFamily="34" charset="0"/>
+          </a:endParaRPr>
+        </a:p>
+        <a:p>
+          <a:pPr marL="0" marR="0" indent="0" algn="l">
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+            <a:spcBef>
+              <a:spcPts val="0"/>
+            </a:spcBef>
+            <a:spcAft>
+              <a:spcPts val="0"/>
+            </a:spcAft>
+          </a:pPr>
+          <a:endParaRPr lang="en-US" sz="1100" b="0" i="0" u="none" strike="noStrike">
+            <a:solidFill>
+              <a:schemeClr val="lt1"/>
+            </a:solidFill>
+            <a:latin typeface="Aptos Narrow" panose="020B0004020202020204" pitchFamily="34" charset="0"/>
+          </a:endParaRPr>
+        </a:p>
+        <a:p>
+          <a:pPr marL="0" marR="0" indent="0" algn="l">
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+            <a:spcBef>
+              <a:spcPts val="0"/>
+            </a:spcBef>
+            <a:spcAft>
+              <a:spcPts val="0"/>
+            </a:spcAft>
+          </a:pPr>
+          <a:endParaRPr lang="en-US" sz="1100" b="0" i="0" u="none" strike="noStrike">
+            <a:solidFill>
+              <a:schemeClr val="lt1"/>
+            </a:solidFill>
+            <a:latin typeface="Aptos Narrow" panose="020B0004020202020204" pitchFamily="34" charset="0"/>
+          </a:endParaRPr>
+        </a:p>
+        <a:p>
+          <a:pPr marL="0" marR="0" indent="0" algn="l">
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+            <a:spcBef>
+              <a:spcPts val="0"/>
+            </a:spcBef>
+            <a:spcAft>
+              <a:spcPts val="0"/>
+            </a:spcAft>
+          </a:pPr>
+          <a:endParaRPr lang="en-US" sz="1100" b="0" i="0" u="none" strike="noStrike">
+            <a:solidFill>
+              <a:schemeClr val="lt1"/>
+            </a:solidFill>
+            <a:latin typeface="Aptos Narrow" panose="020B0004020202020204" pitchFamily="34" charset="0"/>
+          </a:endParaRPr>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing25.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>9525</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>47625</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="2" name="四角形 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B167DCDC-7C12-4973-BF6B-B50D67C51EE7}"/>
+            </a:ext>
+            <a:ext uri="{147F2762-F138-4A5C-976F-8EAC2B608ADB}">
+              <a16:predDERef xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" pred="{15723AC8-7A10-4908-982D-E38FEF435220}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1371600" y="800100"/>
+          <a:ext cx="5495925" cy="847725"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="15000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr spcFirstLastPara="0" wrap="square" lIns="91440" tIns="45720" rIns="91440" bIns="45720" rtlCol="0" anchor="t">
+          <a:noAutofit/>
+        </a:bodyPr>
+        <a:lstStyle>
+          <a:lvl1pPr marL="0" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl1pPr>
+          <a:lvl2pPr marL="457200" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl2pPr>
+          <a:lvl3pPr marL="914400" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl3pPr>
+          <a:lvl4pPr marL="1371600" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl4pPr>
+          <a:lvl5pPr marL="1828800" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl5pPr>
+          <a:lvl6pPr marL="2286000" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl6pPr>
+          <a:lvl7pPr marL="2743200" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl7pPr>
+          <a:lvl8pPr marL="3200400" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl8pPr>
+          <a:lvl9pPr marL="3657600" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl9pPr>
+        </a:lstStyle>
+        <a:p>
+          <a:pPr marL="0" marR="0" indent="0" algn="l">
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+            <a:spcBef>
+              <a:spcPts val="0"/>
+            </a:spcBef>
+            <a:spcAft>
+              <a:spcPts val="0"/>
+            </a:spcAft>
+          </a:pPr>
+          <a:r>
+            <a:rPr lang="en-US" sz="3600" b="0" i="0" u="none" strike="noStrike">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="Aptos Narrow" panose="020B0004020202020204" pitchFamily="34" charset="0"/>
+            </a:rPr>
+            <a:t>StatusGetDAO</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>676275</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>676275</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>28575</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="3" name="四角形 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3ECBA4BE-DEBD-4007-826A-77989BED3754}"/>
+            </a:ext>
+            <a:ext uri="{147F2762-F138-4A5C-976F-8EAC2B608ADB}">
+              <a16:predDERef xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" pred="{B167DCDC-7C12-4973-BF6B-B50D67C51EE7}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1362075" y="1476375"/>
+          <a:ext cx="5486400" cy="4152900"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="accent2"/>
+        </a:solidFill>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="15000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr rot="0" spcFirstLastPara="0" vert="horz" wrap="square" lIns="91440" tIns="45720" rIns="91440" bIns="45720" numCol="1" spcCol="0" rtlCol="0" fromWordArt="0" anchor="t" anchorCtr="0" forceAA="0" compatLnSpc="1">
+          <a:prstTxWarp prst="textNoShape">
+            <a:avLst/>
+          </a:prstTxWarp>
+          <a:noAutofit/>
+        </a:bodyPr>
+        <a:lstStyle>
+          <a:lvl1pPr marL="0" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl1pPr>
+          <a:lvl2pPr marL="457200" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl2pPr>
+          <a:lvl3pPr marL="914400" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl3pPr>
+          <a:lvl4pPr marL="1371600" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl4pPr>
+          <a:lvl5pPr marL="1828800" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl5pPr>
+          <a:lvl6pPr marL="2286000" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl6pPr>
+          <a:lvl7pPr marL="2743200" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl7pPr>
+          <a:lvl8pPr marL="3200400" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl8pPr>
+          <a:lvl9pPr marL="3657600" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl9pPr>
+        </a:lstStyle>
+        <a:p>
+          <a:pPr marL="0" indent="0" algn="l"/>
+          <a:endParaRPr lang="en-US" sz="1100" b="0" i="0" u="none" strike="noStrike">
+            <a:solidFill>
+              <a:schemeClr val="lt1"/>
+            </a:solidFill>
+            <a:latin typeface="Aptos Narrow" panose="020B0004020202020204" pitchFamily="34" charset="0"/>
+          </a:endParaRPr>
+        </a:p>
+        <a:p>
+          <a:pPr marL="0" marR="0" indent="0" algn="l">
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+            <a:spcBef>
+              <a:spcPts val="0"/>
+            </a:spcBef>
+            <a:spcAft>
+              <a:spcPts val="0"/>
+            </a:spcAft>
+          </a:pPr>
+          <a:endParaRPr lang="en-US" sz="1100" b="0" i="0" u="none" strike="noStrike">
+            <a:solidFill>
+              <a:schemeClr val="lt1"/>
+            </a:solidFill>
+            <a:latin typeface="Aptos Narrow" panose="020B0004020202020204" pitchFamily="34" charset="0"/>
+          </a:endParaRPr>
+        </a:p>
+        <a:p>
+          <a:pPr marL="0" indent="0"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="0" i="0" u="none" strike="noStrike">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="Aptos Narrow" panose="020B0004020202020204" pitchFamily="34" charset="0"/>
+            </a:rPr>
+            <a:t>- getStatus(dates : ArrayList&lt;LocalDate&gt;) : ArrayList&lt;String&gt;</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr marL="0" marR="0" indent="0" algn="l">
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+            <a:spcBef>
+              <a:spcPts val="0"/>
+            </a:spcBef>
+            <a:spcAft>
+              <a:spcPts val="0"/>
+            </a:spcAft>
+          </a:pPr>
+          <a:endParaRPr lang="en-US" sz="1100" b="0" i="0" u="none" strike="noStrike">
+            <a:solidFill>
+              <a:schemeClr val="lt1"/>
+            </a:solidFill>
+            <a:latin typeface="Aptos Narrow" panose="020B0004020202020204" pitchFamily="34" charset="0"/>
+          </a:endParaRPr>
+        </a:p>
+        <a:p>
+          <a:pPr marL="0" marR="0" indent="0" algn="l">
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+            <a:spcBef>
+              <a:spcPts val="0"/>
+            </a:spcBef>
+            <a:spcAft>
+              <a:spcPts val="0"/>
+            </a:spcAft>
+          </a:pPr>
+          <a:endParaRPr lang="en-US" sz="1100" b="0" i="0" u="none" strike="noStrike">
+            <a:solidFill>
+              <a:schemeClr val="lt1"/>
+            </a:solidFill>
+            <a:latin typeface="Aptos Narrow" panose="020B0004020202020204" pitchFamily="34" charset="0"/>
+          </a:endParaRPr>
+        </a:p>
+        <a:p>
+          <a:pPr marL="0" marR="0" indent="0" algn="l">
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+            <a:spcBef>
+              <a:spcPts val="0"/>
+            </a:spcBef>
+            <a:spcAft>
+              <a:spcPts val="0"/>
+            </a:spcAft>
+          </a:pPr>
+          <a:endParaRPr lang="en-US" sz="1100" b="0" i="0" u="none" strike="noStrike">
+            <a:solidFill>
+              <a:schemeClr val="lt1"/>
+            </a:solidFill>
+            <a:latin typeface="Aptos Narrow" panose="020B0004020202020204" pitchFamily="34" charset="0"/>
+          </a:endParaRPr>
+        </a:p>
+        <a:p>
+          <a:pPr marL="0" marR="0" indent="0" algn="l">
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+            <a:spcBef>
+              <a:spcPts val="0"/>
+            </a:spcBef>
+            <a:spcAft>
+              <a:spcPts val="0"/>
+            </a:spcAft>
+          </a:pPr>
+          <a:endParaRPr lang="en-US" sz="1100" b="0" i="0" u="none" strike="noStrike">
+            <a:solidFill>
+              <a:schemeClr val="lt1"/>
+            </a:solidFill>
+            <a:latin typeface="Aptos Narrow" panose="020B0004020202020204" pitchFamily="34" charset="0"/>
+          </a:endParaRPr>
+        </a:p>
+        <a:p>
+          <a:pPr marL="0" marR="0" indent="0" algn="l">
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+            <a:spcBef>
+              <a:spcPts val="0"/>
+            </a:spcBef>
+            <a:spcAft>
+              <a:spcPts val="0"/>
+            </a:spcAft>
+          </a:pPr>
+          <a:endParaRPr lang="en-US" sz="1100" b="0" i="0" u="none" strike="noStrike">
+            <a:solidFill>
+              <a:schemeClr val="lt1"/>
+            </a:solidFill>
+            <a:latin typeface="Aptos Narrow" panose="020B0004020202020204" pitchFamily="34" charset="0"/>
+          </a:endParaRPr>
+        </a:p>
+        <a:p>
+          <a:pPr marL="0" marR="0" indent="0" algn="l">
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+            <a:spcBef>
+              <a:spcPts val="0"/>
+            </a:spcBef>
+            <a:spcAft>
+              <a:spcPts val="0"/>
+            </a:spcAft>
+          </a:pPr>
+          <a:endParaRPr lang="en-US" sz="1100" b="0" i="0" u="none" strike="noStrike">
+            <a:solidFill>
+              <a:schemeClr val="lt1"/>
+            </a:solidFill>
+            <a:latin typeface="Aptos Narrow" panose="020B0004020202020204" pitchFamily="34" charset="0"/>
+          </a:endParaRPr>
+        </a:p>
+        <a:p>
+          <a:pPr marL="0" marR="0" indent="0" algn="l">
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+            <a:spcBef>
+              <a:spcPts val="0"/>
+            </a:spcBef>
+            <a:spcAft>
+              <a:spcPts val="0"/>
+            </a:spcAft>
+          </a:pPr>
+          <a:endParaRPr lang="en-US" sz="1100" b="0" i="0" u="none" strike="noStrike">
+            <a:solidFill>
+              <a:schemeClr val="lt1"/>
+            </a:solidFill>
+            <a:latin typeface="Aptos Narrow" panose="020B0004020202020204" pitchFamily="34" charset="0"/>
+          </a:endParaRPr>
+        </a:p>
+        <a:p>
+          <a:pPr marL="0" marR="0" indent="0" algn="l">
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+            <a:spcBef>
+              <a:spcPts val="0"/>
+            </a:spcBef>
+            <a:spcAft>
+              <a:spcPts val="0"/>
+            </a:spcAft>
+          </a:pPr>
+          <a:endParaRPr lang="en-US" sz="1100" b="0" i="0" u="none" strike="noStrike">
+            <a:solidFill>
+              <a:schemeClr val="lt1"/>
+            </a:solidFill>
+            <a:latin typeface="Aptos Narrow" panose="020B0004020202020204" pitchFamily="34" charset="0"/>
+          </a:endParaRPr>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing26.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>9525</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>47625</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="2" name="四角形 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{846DDE59-C8F1-4378-9518-19D8C521E839}"/>
+            </a:ext>
+            <a:ext uri="{147F2762-F138-4A5C-976F-8EAC2B608ADB}">
+              <a16:predDERef xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" pred="{15723AC8-7A10-4908-982D-E38FEF435220}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1371600" y="800100"/>
+          <a:ext cx="5495925" cy="847725"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="15000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr spcFirstLastPara="0" wrap="square" lIns="91440" tIns="45720" rIns="91440" bIns="45720" rtlCol="0" anchor="t">
+          <a:noAutofit/>
+        </a:bodyPr>
+        <a:lstStyle>
+          <a:lvl1pPr marL="0" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl1pPr>
+          <a:lvl2pPr marL="457200" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl2pPr>
+          <a:lvl3pPr marL="914400" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl3pPr>
+          <a:lvl4pPr marL="1371600" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl4pPr>
+          <a:lvl5pPr marL="1828800" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl5pPr>
+          <a:lvl6pPr marL="2286000" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl6pPr>
+          <a:lvl7pPr marL="2743200" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl7pPr>
+          <a:lvl8pPr marL="3200400" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl8pPr>
+          <a:lvl9pPr marL="3657600" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl9pPr>
+        </a:lstStyle>
+        <a:p>
+          <a:pPr marL="0" marR="0" indent="0" algn="l">
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+            <a:spcBef>
+              <a:spcPts val="0"/>
+            </a:spcBef>
+            <a:spcAft>
+              <a:spcPts val="0"/>
+            </a:spcAft>
+          </a:pPr>
+          <a:r>
+            <a:rPr lang="en-US" sz="3600" b="0" i="0" u="none" strike="noStrike">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="Aptos Narrow" panose="020B0004020202020204" pitchFamily="34" charset="0"/>
+            </a:rPr>
+            <a:t>StatusGetServlet</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>676275</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>676275</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>28575</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="3" name="四角形 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{868A0325-DC00-454B-9AFD-35FD3791169A}"/>
+            </a:ext>
+            <a:ext uri="{147F2762-F138-4A5C-976F-8EAC2B608ADB}">
+              <a16:predDERef xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" pred="{846DDE59-C8F1-4378-9518-19D8C521E839}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1362075" y="1476375"/>
+          <a:ext cx="5486400" cy="4152900"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="accent2"/>
+        </a:solidFill>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="15000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr rot="0" spcFirstLastPara="0" vert="horz" wrap="square" lIns="91440" tIns="45720" rIns="91440" bIns="45720" numCol="1" spcCol="0" rtlCol="0" fromWordArt="0" anchor="t" anchorCtr="0" forceAA="0" compatLnSpc="1">
+          <a:prstTxWarp prst="textNoShape">
+            <a:avLst/>
+          </a:prstTxWarp>
+          <a:noAutofit/>
+        </a:bodyPr>
+        <a:lstStyle>
+          <a:lvl1pPr marL="0" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl1pPr>
+          <a:lvl2pPr marL="457200" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl2pPr>
+          <a:lvl3pPr marL="914400" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl3pPr>
+          <a:lvl4pPr marL="1371600" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl4pPr>
+          <a:lvl5pPr marL="1828800" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl5pPr>
+          <a:lvl6pPr marL="2286000" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl6pPr>
+          <a:lvl7pPr marL="2743200" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl7pPr>
+          <a:lvl8pPr marL="3200400" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl8pPr>
+          <a:lvl9pPr marL="3657600" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl9pPr>
+        </a:lstStyle>
+        <a:p>
+          <a:pPr marL="0" indent="0" algn="l"/>
+          <a:endParaRPr lang="en-US" sz="1100" b="0" i="0" u="none" strike="noStrike">
+            <a:solidFill>
+              <a:schemeClr val="lt1"/>
+            </a:solidFill>
+            <a:latin typeface="Aptos Narrow" panose="020B0004020202020204" pitchFamily="34" charset="0"/>
+          </a:endParaRPr>
+        </a:p>
+        <a:p>
+          <a:pPr marL="0" marR="0" indent="0" algn="l">
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+            <a:spcBef>
+              <a:spcPts val="0"/>
+            </a:spcBef>
+            <a:spcAft>
+              <a:spcPts val="0"/>
+            </a:spcAft>
+          </a:pPr>
+          <a:endParaRPr lang="en-US" sz="1100" b="0" i="0" u="none" strike="noStrike">
+            <a:solidFill>
+              <a:schemeClr val="lt1"/>
+            </a:solidFill>
+            <a:latin typeface="+mn-lt"/>
+            <a:ea typeface="+mn-lt"/>
+            <a:cs typeface="+mn-lt"/>
+          </a:endParaRPr>
+        </a:p>
+        <a:p>
+          <a:pPr marL="0" indent="0"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="0" i="0">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-lt"/>
+              <a:cs typeface="+mn-lt"/>
+            </a:rPr>
+            <a:t># doGet(request : HttpServletRequest ,response :  HttpServletResponse) : void</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr marL="0" indent="0"/>
+          <a:endParaRPr lang="en-US" sz="1100" b="0" i="0">
+            <a:solidFill>
+              <a:schemeClr val="lt1"/>
+            </a:solidFill>
+            <a:latin typeface="+mn-lt"/>
+            <a:ea typeface="+mn-lt"/>
+            <a:cs typeface="+mn-lt"/>
+          </a:endParaRPr>
+        </a:p>
+        <a:p>
+          <a:pPr marL="0" indent="0"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="0" i="0">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-lt"/>
+              <a:cs typeface="+mn-lt"/>
+            </a:rPr>
+            <a:t># doPost(request : HttpServletRequest ,response :  HttpServletResponse) : void</a:t>
+          </a:r>
+          <a:endParaRPr lang="en-US" sz="1100" b="0" i="0" u="none" strike="noStrike">
+            <a:solidFill>
+              <a:schemeClr val="lt1"/>
+            </a:solidFill>
+            <a:latin typeface="Aptos Narrow" panose="020B0004020202020204" pitchFamily="34" charset="0"/>
+          </a:endParaRPr>
+        </a:p>
+        <a:p>
+          <a:pPr marL="0" marR="0" indent="0" algn="l">
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+            <a:spcBef>
+              <a:spcPts val="0"/>
+            </a:spcBef>
+            <a:spcAft>
+              <a:spcPts val="0"/>
+            </a:spcAft>
+          </a:pPr>
+          <a:endParaRPr lang="en-US" sz="1100" b="0" i="0" u="none" strike="noStrike">
+            <a:solidFill>
+              <a:schemeClr val="lt1"/>
+            </a:solidFill>
+            <a:latin typeface="Aptos Narrow" panose="020B0004020202020204" pitchFamily="34" charset="0"/>
+          </a:endParaRPr>
+        </a:p>
+        <a:p>
+          <a:pPr marL="0" marR="0" indent="0" algn="l">
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+            <a:spcBef>
+              <a:spcPts val="0"/>
+            </a:spcBef>
+            <a:spcAft>
+              <a:spcPts val="0"/>
+            </a:spcAft>
+          </a:pPr>
+          <a:endParaRPr lang="en-US" sz="1100" b="0" i="0" u="none" strike="noStrike">
+            <a:solidFill>
+              <a:schemeClr val="lt1"/>
+            </a:solidFill>
+            <a:latin typeface="Aptos Narrow" panose="020B0004020202020204" pitchFamily="34" charset="0"/>
+          </a:endParaRPr>
+        </a:p>
+        <a:p>
+          <a:pPr marL="0" marR="0" indent="0" algn="l">
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+            <a:spcBef>
+              <a:spcPts val="0"/>
+            </a:spcBef>
+            <a:spcAft>
+              <a:spcPts val="0"/>
+            </a:spcAft>
+          </a:pPr>
+          <a:endParaRPr lang="en-US" sz="1100" b="0" i="0" u="none" strike="noStrike">
+            <a:solidFill>
+              <a:schemeClr val="lt1"/>
+            </a:solidFill>
+            <a:latin typeface="Aptos Narrow" panose="020B0004020202020204" pitchFamily="34" charset="0"/>
+          </a:endParaRPr>
+        </a:p>
+        <a:p>
+          <a:pPr marL="0" marR="0" indent="0" algn="l">
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+            <a:spcBef>
+              <a:spcPts val="0"/>
+            </a:spcBef>
+            <a:spcAft>
+              <a:spcPts val="0"/>
+            </a:spcAft>
+          </a:pPr>
+          <a:endParaRPr lang="en-US" sz="1100" b="0" i="0" u="none" strike="noStrike">
+            <a:solidFill>
+              <a:schemeClr val="lt1"/>
+            </a:solidFill>
+            <a:latin typeface="Aptos Narrow" panose="020B0004020202020204" pitchFamily="34" charset="0"/>
+          </a:endParaRPr>
+        </a:p>
+        <a:p>
+          <a:pPr marL="0" marR="0" indent="0" algn="l">
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+            <a:spcBef>
+              <a:spcPts val="0"/>
+            </a:spcBef>
+            <a:spcAft>
+              <a:spcPts val="0"/>
+            </a:spcAft>
+          </a:pPr>
+          <a:endParaRPr lang="en-US" sz="1100" b="0" i="0" u="none" strike="noStrike">
+            <a:solidFill>
+              <a:schemeClr val="lt1"/>
+            </a:solidFill>
+            <a:latin typeface="Aptos Narrow" panose="020B0004020202020204" pitchFamily="34" charset="0"/>
+          </a:endParaRPr>
+        </a:p>
+        <a:p>
+          <a:pPr marL="0" marR="0" indent="0" algn="l">
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+            <a:spcBef>
+              <a:spcPts val="0"/>
+            </a:spcBef>
+            <a:spcAft>
+              <a:spcPts val="0"/>
+            </a:spcAft>
+          </a:pPr>
+          <a:endParaRPr lang="en-US" sz="1100" b="0" i="0" u="none" strike="noStrike">
+            <a:solidFill>
+              <a:schemeClr val="lt1"/>
+            </a:solidFill>
+            <a:latin typeface="Aptos Narrow" panose="020B0004020202020204" pitchFamily="34" charset="0"/>
+          </a:endParaRPr>
+        </a:p>
+        <a:p>
+          <a:pPr marL="0" marR="0" indent="0" algn="l">
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+            <a:spcBef>
+              <a:spcPts val="0"/>
+            </a:spcBef>
+            <a:spcAft>
+              <a:spcPts val="0"/>
+            </a:spcAft>
+          </a:pPr>
+          <a:endParaRPr lang="en-US" sz="1100" b="0" i="0" u="none" strike="noStrike">
+            <a:solidFill>
+              <a:schemeClr val="lt1"/>
+            </a:solidFill>
+            <a:latin typeface="Aptos Narrow" panose="020B0004020202020204" pitchFamily="34" charset="0"/>
+          </a:endParaRPr>
+        </a:p>
+        <a:p>
+          <a:pPr marL="0" marR="0" indent="0" algn="l">
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+            <a:spcBef>
+              <a:spcPts val="0"/>
+            </a:spcBef>
+            <a:spcAft>
+              <a:spcPts val="0"/>
+            </a:spcAft>
+          </a:pPr>
+          <a:endParaRPr lang="en-US" sz="1100" b="0" i="0" u="none" strike="noStrike">
+            <a:solidFill>
+              <a:schemeClr val="lt1"/>
+            </a:solidFill>
+            <a:latin typeface="Aptos Narrow" panose="020B0004020202020204" pitchFamily="34" charset="0"/>
+          </a:endParaRPr>
+        </a:p>
+        <a:p>
+          <a:pPr marL="0" marR="0" indent="0" algn="l">
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+            <a:spcBef>
+              <a:spcPts val="0"/>
+            </a:spcBef>
+            <a:spcAft>
+              <a:spcPts val="0"/>
+            </a:spcAft>
+          </a:pPr>
+          <a:endParaRPr lang="en-US" sz="1100" b="0" i="0" u="none" strike="noStrike">
+            <a:solidFill>
+              <a:schemeClr val="lt1"/>
+            </a:solidFill>
+            <a:latin typeface="Aptos Narrow" panose="020B0004020202020204" pitchFamily="34" charset="0"/>
+          </a:endParaRPr>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing27.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>9525</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>47625</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="2" name="四角形 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9C1FCEB0-4A05-461F-993E-DA01BC2676A0}"/>
+            </a:ext>
+            <a:ext uri="{147F2762-F138-4A5C-976F-8EAC2B608ADB}">
+              <a16:predDERef xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" pred="{15723AC8-7A10-4908-982D-E38FEF435220}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1371600" y="800100"/>
+          <a:ext cx="5495925" cy="847725"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="15000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr spcFirstLastPara="0" wrap="square" lIns="91440" tIns="45720" rIns="91440" bIns="45720" rtlCol="0" anchor="t">
+          <a:noAutofit/>
+        </a:bodyPr>
+        <a:lstStyle>
+          <a:lvl1pPr marL="0" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl1pPr>
+          <a:lvl2pPr marL="457200" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl2pPr>
+          <a:lvl3pPr marL="914400" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl3pPr>
+          <a:lvl4pPr marL="1371600" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl4pPr>
+          <a:lvl5pPr marL="1828800" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl5pPr>
+          <a:lvl6pPr marL="2286000" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl6pPr>
+          <a:lvl7pPr marL="2743200" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl7pPr>
+          <a:lvl8pPr marL="3200400" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl8pPr>
+          <a:lvl9pPr marL="3657600" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl9pPr>
+        </a:lstStyle>
+        <a:p>
+          <a:pPr marL="0" marR="0" indent="0" algn="l">
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+            <a:spcBef>
+              <a:spcPts val="0"/>
+            </a:spcBef>
+            <a:spcAft>
+              <a:spcPts val="0"/>
+            </a:spcAft>
+          </a:pPr>
+          <a:r>
+            <a:rPr lang="en-US" sz="3600" b="0" i="0" u="none" strike="noStrike">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="Aptos Narrow" panose="020B0004020202020204" pitchFamily="34" charset="0"/>
+            </a:rPr>
+            <a:t>WeeksGet</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>676275</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>676275</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>28575</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="3" name="四角形 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B889F2CE-7CA8-416D-8EEC-A5FC9B563F34}"/>
+            </a:ext>
+            <a:ext uri="{147F2762-F138-4A5C-976F-8EAC2B608ADB}">
+              <a16:predDERef xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" pred="{9C1FCEB0-4A05-461F-993E-DA01BC2676A0}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1362075" y="1476375"/>
+          <a:ext cx="5486400" cy="4152900"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="accent2"/>
+        </a:solidFill>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="15000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr rot="0" spcFirstLastPara="0" vert="horz" wrap="square" lIns="91440" tIns="45720" rIns="91440" bIns="45720" numCol="1" spcCol="0" rtlCol="0" fromWordArt="0" anchor="t" anchorCtr="0" forceAA="0" compatLnSpc="1">
+          <a:prstTxWarp prst="textNoShape">
+            <a:avLst/>
+          </a:prstTxWarp>
+          <a:noAutofit/>
+        </a:bodyPr>
+        <a:lstStyle>
+          <a:lvl1pPr marL="0" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl1pPr>
+          <a:lvl2pPr marL="457200" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl2pPr>
+          <a:lvl3pPr marL="914400" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl3pPr>
+          <a:lvl4pPr marL="1371600" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl4pPr>
+          <a:lvl5pPr marL="1828800" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl5pPr>
+          <a:lvl6pPr marL="2286000" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl6pPr>
+          <a:lvl7pPr marL="2743200" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl7pPr>
+          <a:lvl8pPr marL="3200400" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl8pPr>
+          <a:lvl9pPr marL="3657600" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl9pPr>
+        </a:lstStyle>
+        <a:p>
+          <a:pPr marL="0" indent="0" algn="l"/>
+          <a:endParaRPr lang="en-US" sz="1100" b="0" i="0" u="none" strike="noStrike">
+            <a:solidFill>
+              <a:schemeClr val="lt1"/>
+            </a:solidFill>
+            <a:latin typeface="+mn-lt"/>
+            <a:ea typeface="+mn-lt"/>
+            <a:cs typeface="+mn-lt"/>
+          </a:endParaRPr>
+        </a:p>
+        <a:p>
+          <a:pPr marL="0" marR="0" indent="0" algn="l">
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+            <a:spcBef>
+              <a:spcPts val="0"/>
+            </a:spcBef>
+            <a:spcAft>
+              <a:spcPts val="0"/>
+            </a:spcAft>
+          </a:pPr>
+          <a:endParaRPr lang="en-US" sz="1100" b="0" i="0" u="none" strike="noStrike">
+            <a:solidFill>
+              <a:schemeClr val="lt1"/>
+            </a:solidFill>
+            <a:latin typeface="Aptos Narrow" panose="020B0004020202020204" pitchFamily="34" charset="0"/>
+          </a:endParaRPr>
+        </a:p>
+        <a:p>
+          <a:pPr marL="0" indent="0"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="0" i="0" u="none" strike="noStrike">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="Aptos Narrow" panose="020B0004020202020204" pitchFamily="34" charset="0"/>
+            </a:rPr>
+            <a:t>- getWeeks(todayWeek : DayOfWeek) : ArrayList&lt;String&gt;</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr marL="0" marR="0" indent="0" algn="l">
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+            <a:spcBef>
+              <a:spcPts val="0"/>
+            </a:spcBef>
+            <a:spcAft>
+              <a:spcPts val="0"/>
+            </a:spcAft>
+          </a:pPr>
+          <a:endParaRPr lang="en-US" sz="1100" b="0" i="0" u="none" strike="noStrike">
+            <a:solidFill>
+              <a:schemeClr val="lt1"/>
+            </a:solidFill>
+            <a:latin typeface="Aptos Narrow" panose="020B0004020202020204" pitchFamily="34" charset="0"/>
+          </a:endParaRPr>
+        </a:p>
+        <a:p>
+          <a:pPr marL="0" marR="0" indent="0" algn="l">
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+            <a:spcBef>
+              <a:spcPts val="0"/>
+            </a:spcBef>
+            <a:spcAft>
+              <a:spcPts val="0"/>
+            </a:spcAft>
+          </a:pPr>
+          <a:endParaRPr lang="en-US" sz="1100" b="0" i="0" u="none" strike="noStrike">
+            <a:solidFill>
+              <a:schemeClr val="lt1"/>
+            </a:solidFill>
+            <a:latin typeface="Aptos Narrow" panose="020B0004020202020204" pitchFamily="34" charset="0"/>
+          </a:endParaRPr>
+        </a:p>
+        <a:p>
+          <a:pPr marL="0" marR="0" indent="0" algn="l">
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+            <a:spcBef>
+              <a:spcPts val="0"/>
+            </a:spcBef>
+            <a:spcAft>
+              <a:spcPts val="0"/>
+            </a:spcAft>
+          </a:pPr>
+          <a:endParaRPr lang="en-US" sz="1100" b="0" i="0" u="none" strike="noStrike">
+            <a:solidFill>
+              <a:schemeClr val="lt1"/>
+            </a:solidFill>
+            <a:latin typeface="Aptos Narrow" panose="020B0004020202020204" pitchFamily="34" charset="0"/>
+          </a:endParaRPr>
+        </a:p>
+        <a:p>
+          <a:pPr marL="0" marR="0" indent="0" algn="l">
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+            <a:spcBef>
+              <a:spcPts val="0"/>
+            </a:spcBef>
+            <a:spcAft>
+              <a:spcPts val="0"/>
+            </a:spcAft>
+          </a:pPr>
+          <a:endParaRPr lang="en-US" sz="1100" b="0" i="0" u="none" strike="noStrike">
+            <a:solidFill>
+              <a:schemeClr val="lt1"/>
+            </a:solidFill>
+            <a:latin typeface="Aptos Narrow" panose="020B0004020202020204" pitchFamily="34" charset="0"/>
+          </a:endParaRPr>
+        </a:p>
+        <a:p>
+          <a:pPr marL="0" marR="0" indent="0" algn="l">
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+            <a:spcBef>
+              <a:spcPts val="0"/>
+            </a:spcBef>
+            <a:spcAft>
+              <a:spcPts val="0"/>
+            </a:spcAft>
+          </a:pPr>
+          <a:endParaRPr lang="en-US" sz="1100" b="0" i="0" u="none" strike="noStrike">
+            <a:solidFill>
+              <a:schemeClr val="lt1"/>
+            </a:solidFill>
+            <a:latin typeface="Aptos Narrow" panose="020B0004020202020204" pitchFamily="34" charset="0"/>
+          </a:endParaRPr>
+        </a:p>
+        <a:p>
+          <a:pPr marL="0" marR="0" indent="0" algn="l">
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+            <a:spcBef>
+              <a:spcPts val="0"/>
+            </a:spcBef>
+            <a:spcAft>
+              <a:spcPts val="0"/>
+            </a:spcAft>
+          </a:pPr>
+          <a:endParaRPr lang="en-US" sz="1100" b="0" i="0" u="none" strike="noStrike">
+            <a:solidFill>
+              <a:schemeClr val="lt1"/>
+            </a:solidFill>
+            <a:latin typeface="Aptos Narrow" panose="020B0004020202020204" pitchFamily="34" charset="0"/>
+          </a:endParaRPr>
+        </a:p>
+        <a:p>
+          <a:pPr marL="0" marR="0" indent="0" algn="l">
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+            <a:spcBef>
+              <a:spcPts val="0"/>
+            </a:spcBef>
+            <a:spcAft>
+              <a:spcPts val="0"/>
+            </a:spcAft>
+          </a:pPr>
+          <a:endParaRPr lang="en-US" sz="1100" b="0" i="0" u="none" strike="noStrike">
+            <a:solidFill>
+              <a:schemeClr val="lt1"/>
+            </a:solidFill>
+            <a:latin typeface="Aptos Narrow" panose="020B0004020202020204" pitchFamily="34" charset="0"/>
+          </a:endParaRPr>
+        </a:p>
+        <a:p>
+          <a:pPr marL="0" marR="0" indent="0" algn="l">
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+            <a:spcBef>
+              <a:spcPts val="0"/>
+            </a:spcBef>
+            <a:spcAft>
+              <a:spcPts val="0"/>
+            </a:spcAft>
+          </a:pPr>
+          <a:endParaRPr lang="en-US" sz="1100" b="0" i="0" u="none" strike="noStrike">
+            <a:solidFill>
+              <a:schemeClr val="lt1"/>
+            </a:solidFill>
+            <a:latin typeface="Aptos Narrow" panose="020B0004020202020204" pitchFamily="34" charset="0"/>
+          </a:endParaRPr>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing28.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>9525</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>47625</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="2" name="四角形 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{62D721A1-14B6-419C-825A-BB043EBCFB7A}"/>
+            </a:ext>
+            <a:ext uri="{147F2762-F138-4A5C-976F-8EAC2B608ADB}">
+              <a16:predDERef xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" pred="{15723AC8-7A10-4908-982D-E38FEF435220}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1371600" y="800100"/>
+          <a:ext cx="5495925" cy="847725"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="15000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr spcFirstLastPara="0" wrap="square" lIns="91440" tIns="45720" rIns="91440" bIns="45720" rtlCol="0" anchor="t">
+          <a:noAutofit/>
+        </a:bodyPr>
+        <a:lstStyle>
+          <a:lvl1pPr marL="0" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl1pPr>
+          <a:lvl2pPr marL="457200" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl2pPr>
+          <a:lvl3pPr marL="914400" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl3pPr>
+          <a:lvl4pPr marL="1371600" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl4pPr>
+          <a:lvl5pPr marL="1828800" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl5pPr>
+          <a:lvl6pPr marL="2286000" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl6pPr>
+          <a:lvl7pPr marL="2743200" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl7pPr>
+          <a:lvl8pPr marL="3200400" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl8pPr>
+          <a:lvl9pPr marL="3657600" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl9pPr>
+        </a:lstStyle>
+        <a:p>
+          <a:pPr marL="0" marR="0" indent="0" algn="l">
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+            <a:spcBef>
+              <a:spcPts val="0"/>
+            </a:spcBef>
+            <a:spcAft>
+              <a:spcPts val="0"/>
+            </a:spcAft>
+          </a:pPr>
+          <a:r>
+            <a:rPr lang="en-US" sz="3600" b="0" i="0" u="none" strike="noStrike">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="Aptos Narrow" panose="020B0004020202020204" pitchFamily="34" charset="0"/>
+            </a:rPr>
+            <a:t>DatesGet</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>676275</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>676275</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>28575</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="3" name="四角形 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E3C818FB-7A98-4946-B7AF-AFB57A8B959D}"/>
+            </a:ext>
+            <a:ext uri="{147F2762-F138-4A5C-976F-8EAC2B608ADB}">
+              <a16:predDERef xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" pred="{62D721A1-14B6-419C-825A-BB043EBCFB7A}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1362075" y="1476375"/>
+          <a:ext cx="5486400" cy="4152900"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="accent2"/>
+        </a:solidFill>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="15000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr rot="0" spcFirstLastPara="0" vert="horz" wrap="square" lIns="91440" tIns="45720" rIns="91440" bIns="45720" numCol="1" spcCol="0" rtlCol="0" fromWordArt="0" anchor="t" anchorCtr="0" forceAA="0" compatLnSpc="1">
+          <a:prstTxWarp prst="textNoShape">
+            <a:avLst/>
+          </a:prstTxWarp>
+          <a:noAutofit/>
+        </a:bodyPr>
+        <a:lstStyle>
+          <a:lvl1pPr marL="0" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl1pPr>
+          <a:lvl2pPr marL="457200" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl2pPr>
+          <a:lvl3pPr marL="914400" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl3pPr>
+          <a:lvl4pPr marL="1371600" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl4pPr>
+          <a:lvl5pPr marL="1828800" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl5pPr>
+          <a:lvl6pPr marL="2286000" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl6pPr>
+          <a:lvl7pPr marL="2743200" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl7pPr>
+          <a:lvl8pPr marL="3200400" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl8pPr>
+          <a:lvl9pPr marL="3657600" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl9pPr>
+        </a:lstStyle>
+        <a:p>
+          <a:pPr marL="0" indent="0" algn="l"/>
+          <a:endParaRPr lang="en-US" sz="1100" b="0" i="0" u="none" strike="noStrike">
+            <a:solidFill>
+              <a:schemeClr val="lt1"/>
+            </a:solidFill>
+            <a:latin typeface="Aptos Narrow" panose="020B0004020202020204" pitchFamily="34" charset="0"/>
+          </a:endParaRPr>
+        </a:p>
+        <a:p>
+          <a:pPr marL="0" marR="0" indent="0" algn="l">
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+            <a:spcBef>
+              <a:spcPts val="0"/>
+            </a:spcBef>
+            <a:spcAft>
+              <a:spcPts val="0"/>
+            </a:spcAft>
+          </a:pPr>
+          <a:endParaRPr lang="en-US" sz="1100" b="0" i="0" u="none" strike="noStrike">
+            <a:solidFill>
+              <a:schemeClr val="lt1"/>
+            </a:solidFill>
+            <a:latin typeface="Aptos Narrow" panose="020B0004020202020204" pitchFamily="34" charset="0"/>
+          </a:endParaRPr>
+        </a:p>
+        <a:p>
+          <a:pPr marL="0" indent="0"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="0" i="0" u="none" strike="noStrike">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="Aptos Narrow" panose="020B0004020202020204" pitchFamily="34" charset="0"/>
+            </a:rPr>
+            <a:t>- getDates(today : LocalDate) : ArrayList&lt;LocalDate&gt;</a:t>
+          </a:r>
         </a:p>
         <a:p>
           <a:pPr marL="0" marR="0" indent="0" algn="l">
@@ -11186,6 +13386,39 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A132E543-2CC7-4800-B3E9-A1B4345EB203}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.75"/>
+  <sheetData/>
+  <phoneticPr fontId="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{162AA59B-CAC8-4B3C-8F31-2455B8C88E34}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.75"/>
+  <sheetData/>
+  <phoneticPr fontId="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8B6B4758-7A84-47A0-BA34-81FBCD200257}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.75"/>
+  <sheetData/>
+  <phoneticPr fontId="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E7027D6D-8678-4A17-A748-A2602CED5D96}">
   <dimension ref="C5:O11"/>
@@ -11220,6 +13453,17 @@
     <mergeCell ref="L11:O11"/>
   </mergeCells>
   <phoneticPr fontId="8"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D4F506AF-BC37-4BE1-9D8C-71052C40479A}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.75"/>
+  <sheetData/>
+  <phoneticPr fontId="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>